<commit_message>
WebDriver Day-13 & TestNG Day-5
</commit_message>
<xml_diff>
--- a/TestData2/Data.xlsx
+++ b/TestData2/Data.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28623"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ganes\OneDrive\Desktop\Learning\WeekendDec24-25\MavenSelenium\TestData\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ganes\OneDrive\Desktop\Learning\WeekendDec24-25\MavenSelenium\TestData2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56C09AC4-B095-4FF6-81B6-48943392C773}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E41766AB-B938-4798-8EA2-A5B0723F6697}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BookData" sheetId="1" r:id="rId1"/>
+    <sheet name="userdata" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="18">
   <si>
     <t>BookName</t>
   </si>
@@ -58,13 +59,34 @@
   </si>
   <si>
     <t>Naveen</t>
+  </si>
+  <si>
+    <t>UserName</t>
+  </si>
+  <si>
+    <t>Password</t>
+  </si>
+  <si>
+    <t>Admin</t>
+  </si>
+  <si>
+    <t>admin123</t>
+  </si>
+  <si>
+    <t>Smita</t>
+  </si>
+  <si>
+    <t>test123</t>
+  </si>
+  <si>
+    <t>Parag</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -90,6 +112,28 @@
     <font>
       <b/>
       <sz val="20"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="26"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="26"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="24"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -131,11 +175,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -482,4 +529,66 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{89B6BE54-1050-44AB-A29B-C12EA1D66786}">
+  <dimension ref="A1:B6"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="30.109375" customWidth="1"/>
+    <col min="2" max="2" width="30.33203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" s="3" customFormat="1" ht="33.6" x14ac:dyDescent="0.65">
+      <c r="A1" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" ht="33.6" x14ac:dyDescent="0.65">
+      <c r="A2" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="33.6" x14ac:dyDescent="0.65">
+      <c r="A3" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="33.6" x14ac:dyDescent="0.65">
+      <c r="A4" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" ht="33.6" x14ac:dyDescent="0.65">
+      <c r="A5" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" ht="31.2" x14ac:dyDescent="0.6">
+      <c r="A6" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>14</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>